<commit_message>
Add formatted cheap MVP BOM spreadsheet.
</commit_message>
<xml_diff>
--- a/docs/bom_mvp_barato.xlsx
+++ b/docs/bom_mvp_barato.xlsx
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;MXN &quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -39,11 +40,11 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00C2410C"/>
+      <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00C2410C"/>
-      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
@@ -112,8 +113,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -124,7 +125,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -133,8 +134,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -501,167 +502,202 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OSMO / Seneca — MVP BARATO (fingertip-only, 1 glove)</t>
+          <t>MVP BARATO — fingertip-only OSMO (1 glove)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>5 taxels (no palm). No Seneca cams. No TagConnect. Clone ST-Link. Tec magnetizer. MQFP price = placeholder until quote.</t>
+          <t>5 taxels · no palm · no cams · clone ST-Link · SWD header · Tec magnetizer · MQFP quote placeholder</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>TOTAL USD</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3477</v>
+        <v>627</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Est. MXN landed</t>
+          <t>Est. MXN</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>79585</v>
+        <v>14035</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>If MQFP quote is $0 sample / cheaper</t>
+          <t>If MQFP sample /$0</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>3327</v>
+        <v>477</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>What we cut vs full BOM</t>
+          <t>vs full ~$1400</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>• Palm sensors (7 boards) → save ~$154 PCBA</t>
+          <t>• No palm → −~$150</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>• Seneca head+wrist cams → save ~$230</t>
+          <t>• No Seneca cams → −~$230</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>• TagConnect → save ~$45 (use $2 SWD header)</t>
+          <t>• No TagConnect/V3/flux/iron → −~$150</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>• Official ST-Link V3 + Chip Quik flux + iron → save ~$100+</t>
+          <t>• Cheaper MuMetal + 1 Sil-Poxy → −~$80</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>• 2nd Sil-Poxy + extras → save ~$50</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>• MuMetal full premium sheet → cheaper cut/share ~$40</t>
+          <t>• → ~$627</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Unit USD</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Ext USD</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Est MXN</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Buy from</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Unit USD</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Ext USD</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Est MXN</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Buy from</t>
-        </is>
-      </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>MCU board PCBA</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>85</v>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>85</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>1955</v>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>JLCPCB/PCBWay</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>1 board enough</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
@@ -670,11 +706,11 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>MCU board PCBA</t>
+          <t>Sensor board PCBA (fingertip only)</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
@@ -682,13 +718,13 @@
         </is>
       </c>
       <c r="F16" s="11" t="n">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="G16" s="11" t="n">
-        <v>85</v>
+        <v>154</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>1955</v>
+        <v>3542</v>
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
@@ -697,64 +733,64 @@
       </c>
       <c r="J16" s="9" t="inlineStr">
         <is>
-          <t>1 board is enough for MVP</t>
+          <t>5 fingers + 2 spare. No palm.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>PCB</t>
+        <v>3</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Magnetics</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Sensor board PCBA (fingertip only)</t>
+          <t>MuMetal small sheet / scrap</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="F17" s="11" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>154</v>
+        <v>40</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>3542</v>
+        <v>920</v>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>JLCPCB/PCBWay</t>
+          <t>DigiKey/Amazon+forwarder</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>5 fingers + 2 spare. Skip palm sensors.</t>
+          <t>Only 5–7 pcs 11×12mm</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Magnetics</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>MuMetal — buy smallest sheet / scrap cut</t>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>MQFP-15-7 powder (20g lot)</t>
         </is>
       </c>
       <c r="D18" s="9" t="n">
@@ -762,74 +798,70 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>sheet</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="F18" s="11" t="n">
-        <v>40</v>
+        <v>150</v>
       </c>
       <c r="G18" s="11" t="n">
-        <v>40</v>
+        <v>150</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>920</v>
+        <v>3450</v>
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>DigiKey/Amazon/forwarder</t>
+          <t>Magnequench quote</t>
         </is>
       </c>
       <c r="J18" s="9" t="inlineStr">
         <is>
-          <t>Need only 5–7 pcs 11×12mm. Split sheet with another lab if possible.</t>
+          <t>PLACEHOLDER until quote. Ask min sample. NOT MQP.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Magnetics</t>
-        </is>
-      </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>MQFP-15-7 powder</t>
+          <t>Silicone</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Ecoflex 00-30 trial kit</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>kit</t>
         </is>
       </c>
       <c r="F19" s="11" t="n">
-        <v>150</v>
+        <v>36</v>
       </c>
       <c r="G19" s="11" t="n">
-        <v>3000</v>
+        <v>36</v>
       </c>
       <c r="H19" s="12" t="n">
-        <v>69000</v>
+        <v>756</v>
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Magnequench quote</t>
-        </is>
-      </c>
-      <c r="J19" s="9" t="inlineStr">
-        <is>
-          <t>Placeholder until quote. Ask for smallest sample/MOQ.</t>
-        </is>
-      </c>
+          <t>Amazon.com.mx</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
@@ -838,7 +870,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Ecoflex 00-30 trial kit</t>
+          <t>Sil-Poxy 3 oz</t>
         </is>
       </c>
       <c r="D20" s="9" t="n">
@@ -846,37 +878,41 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>kit</t>
+          <t>tube</t>
         </is>
       </c>
       <c r="F20" s="11" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G20" s="11" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H20" s="12" t="n">
-        <v>756</v>
+        <v>693</v>
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
           <t>Amazon.com.mx</t>
         </is>
       </c>
-      <c r="J20" s="9" t="inlineStr"/>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>One tube</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Silicone</t>
+          <t>Wiring</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Sil-Poxy 3 oz</t>
+          <t>28 AWG enamel wire</t>
         </is>
       </c>
       <c r="D21" s="9" t="n">
@@ -884,17 +920,17 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>tube</t>
+          <t>spool</t>
         </is>
       </c>
       <c r="F21" s="11" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="H21" s="12" t="n">
-        <v>693</v>
+        <v>189</v>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
@@ -903,102 +939,98 @@
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>One tube for MVP</t>
+          <t>Skip Maeden</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Wiring</t>
+          <t>Glove</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>28 AWG enamel magnet wire</t>
+          <t>Beige thin gloves</t>
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>spool</t>
+          <t>pair</t>
         </is>
       </c>
       <c r="F22" s="11" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G22" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H22" s="12" t="n">
-        <v>189</v>
+        <v>168</v>
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Amazon.com.mx</t>
-        </is>
-      </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>Skip Maeden tinsel</t>
-        </is>
-      </c>
+          <t>Amazon.com.mx / ML</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Glove</t>
+          <t>Consumable</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Beige thin gloves</t>
+          <t>Kapton tape</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>pair</t>
+          <t>roll</t>
         </is>
       </c>
       <c r="F23" s="11" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>168</v>
+        <v>210</v>
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Amazon.com.mx / ML</t>
+          <t>Amazon.com.mx</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Programming</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Kapton tape</t>
+          <t>ST-Link V2 clone</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
@@ -1006,28 +1038,32 @@
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>roll</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="F24" s="11" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G24" s="11" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H24" s="12" t="n">
-        <v>210</v>
+        <v>176</v>
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Amazon.com.mx</t>
-        </is>
-      </c>
-      <c r="J24" s="9" t="inlineStr"/>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>Official V3MINIE=$25 if preferred</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
@@ -1036,7 +1072,7 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>ST-Link V2 clone OR V3MINIE</t>
+          <t>SWD header 1.27mm + jumpers</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
@@ -1044,41 +1080,41 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>set</t>
         </is>
       </c>
       <c r="F25" s="11" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H25" s="12" t="n">
-        <v>176</v>
+        <v>44</v>
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Mercado Libre / Mouser</t>
+          <t>Steren / ML</t>
         </is>
       </c>
       <c r="J25" s="9" t="inlineStr">
         <is>
-          <t>Clone OK for bring-up ($5–12). Official V3MINIE = $25.</t>
+          <t>Skip TagConnect $45</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Programming</t>
+          <t>Cable</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>1.27mm SWD header + Dupont</t>
+          <t>USB-C data cable</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
@@ -1086,70 +1122,66 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="F26" s="11" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H26" s="12" t="n">
-        <v>44</v>
+        <v>168</v>
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>Mercado Libre / Steren</t>
-        </is>
-      </c>
-      <c r="J26" s="9" t="inlineStr">
-        <is>
-          <t>Skip TagConnect ($45)</t>
-        </is>
-      </c>
+          <t>Amazon.com.mx</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Solder + basic flux</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Cable</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>USB-C data cable</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="n">
-        <v>8</v>
-      </c>
       <c r="G27" s="11" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H27" s="12" t="n">
-        <v>168</v>
+        <v>252</v>
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>Amazon.com.mx</t>
+          <t>Steren</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
@@ -1158,7 +1190,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Solder + basic flux paste</t>
+          <t>Multimeter</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
@@ -1166,32 +1198,32 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="F28" s="11" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G28" s="11" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H28" s="12" t="n">
-        <v>252</v>
+        <v>0</v>
       </c>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>Steren / Amazon.com.mx</t>
+          <t>Borrow</t>
         </is>
       </c>
       <c r="J28" s="9" t="inlineStr">
         <is>
-          <t>Skip Chip Quik $40</t>
+          <t>Buy ~$18 if needed</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
@@ -1200,7 +1232,7 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Multimeter (borrow OK)</t>
+          <t>Gram scale 0.1g</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
@@ -1212,66 +1244,62 @@
         </is>
       </c>
       <c r="F29" s="11" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G29" s="11" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H29" s="12" t="n">
-        <v>0</v>
+        <v>252</v>
       </c>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>Borrow / Steren</t>
-        </is>
-      </c>
-      <c r="J29" s="9" t="inlineStr">
-        <is>
-          <t>Put $18 if you must buy</t>
-        </is>
-      </c>
+          <t>Amazon.com.mx</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Cups, sticks, cotton, sandpaper, knife</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>kit</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Tool</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Gram scale 0.1g</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="F30" s="11" t="n">
-        <v>12</v>
-      </c>
       <c r="G30" s="11" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H30" s="12" t="n">
-        <v>252</v>
+        <v>315</v>
       </c>
       <c r="I30" s="9" t="inlineStr">
         <is>
-          <t>Amazon.com.mx</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="J30" s="9" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
@@ -1280,7 +1308,7 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Cups, sticks, cotton tips, sandpaper, knife</t>
+          <t>Mold release spray</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
@@ -1288,7 +1316,7 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>kit</t>
+          <t>can</t>
         </is>
       </c>
       <c r="F31" s="11" t="n">
@@ -1302,23 +1330,23 @@
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t>Local / farmacia</t>
+          <t>Amazon.com.mx</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Tool</t>
+          <t>Fab</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Mold release spray</t>
+          <t>Resin molds fingertips only</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
@@ -1326,37 +1354,37 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>can</t>
+          <t>set</t>
         </is>
       </c>
       <c r="F32" s="11" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G32" s="11" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H32" s="12" t="n">
-        <v>315</v>
+        <v>630</v>
       </c>
       <c r="I32" s="9" t="inlineStr">
         <is>
-          <t>Amazon.com.mx</t>
+          <t>MTY print shop</t>
         </is>
       </c>
       <c r="J32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Fab</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Resin molds fingertips only</t>
+          <t>Pulse magnetizer access</t>
         </is>
       </c>
       <c r="D33" s="9" t="n">
@@ -1364,41 +1392,41 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>access</t>
         </is>
       </c>
       <c r="F33" s="11" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G33" s="11" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H33" s="12" t="n">
-        <v>630</v>
+        <v>0</v>
       </c>
       <c r="I33" s="9" t="inlineStr">
         <is>
-          <t>Local MTY print</t>
+          <t>Tec lab</t>
         </is>
       </c>
       <c r="J33" s="9" t="inlineStr">
         <is>
-          <t>No palm molds</t>
+          <t>Must confirm before build</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Host</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Pulse magnetizer access</t>
+          <t>Linux laptop</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
@@ -1406,7 +1434,7 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>access</t>
+          <t>ea</t>
         </is>
       </c>
       <c r="F34" s="11" t="n">
@@ -1420,76 +1448,30 @@
       </c>
       <c r="I34" s="9" t="inlineStr">
         <is>
-          <t>Tec lab</t>
-        </is>
-      </c>
-      <c r="J34" s="9" t="inlineStr">
-        <is>
-          <t>BLOCKER if no access — then quote Magnet-Physik</t>
-        </is>
-      </c>
+          <t>Owned</t>
+        </is>
+      </c>
+      <c r="J34" s="9" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>Host</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Existing Linux laptop</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="F35" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="9" t="inlineStr">
-        <is>
-          <t>Owned</t>
-        </is>
-      </c>
-      <c r="J35" s="9" t="inlineStr">
-        <is>
-          <t>ROS2 later</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="n"/>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="A35" s="3" t="n"/>
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n"/>
-      <c r="G36" s="14" t="n">
-        <v>3477</v>
-      </c>
-      <c r="H36" s="15" t="n">
-        <v>79585</v>
-      </c>
-      <c r="I36" s="3" t="n"/>
-      <c r="J36" s="3" t="n"/>
+      <c r="D35" s="3" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+      <c r="G35" s="14" t="n">
+        <v>627</v>
+      </c>
+      <c r="H35" s="15" t="n">
+        <v>14035</v>
+      </c>
+      <c r="I35" s="3" t="n"/>
+      <c r="J35" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1505,41 +1487,41 @@
   <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="95" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Orden de compra MVP</t>
+          <t>Orden de compra</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Email Magnequench MQFP-15-7 — pide sample/MOQ mínimo (NO MQP).</t>
+          <t>1. Magnequench MQFP-15-7 sample/quote (NOT MQP).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. Cotiza PCBA: 1–2 MCU + 7 sensor boards en JLCPCB/PCBWay.</t>
+          <t>2. JLCPCB/PCBWay: 1–2 MCU + 7 sensor PCBA.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Confirma magnetizer en Tec (gratis) ANTES de curar skins.</t>
+          <t>3. Confirma magnetizer Tec antes de skins.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4. Amazon MX: Ecoflex, Sil-Poxy×1, wire, gloves, Kapton, USB, scale, mold release.</t>
+          <t>4. Amazon MX: Ecoflex, Sil-Poxy, wire, gloves, Kapton, USB, scale, mold release.</t>
         </is>
       </c>
     </row>
@@ -1553,14 +1535,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6. MuMetal: sheet chica o scrap; corta 7 piezas.</t>
+          <t>6. MuMetal lote chico para 7 piezas.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7. NO compres cámaras Seneca todavía — usa celular para pipeline.</t>
+          <t>7. Cámaras después — celular para software.</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1552,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Success criteria MVP: 5 fingertips stream mag+IMU over USB; 1 wiping demo recorded.</t>
+          <t>Done: 5 fingertips stream USB + 1 demo corta.</t>
         </is>
       </c>
     </row>

</xml_diff>